<commit_message>
Support 'Areas' sheet and enhance dashboards
Load the 'Areas' sheet from Plan de retos.xlsx and thread it through data loaders and renderers. Update _load_plan_retos_data and related callers to return an areas_df (fallback to empty DF on errors). Use Areas data in chip metrics (show total Áreas con Retos) and in Consolidado summary text; adjust unit labels and always show the sunburst when objectives exist. In resumen_por_proceso.py prefer the 'Proceso' column for grouping when present, add a comparison bar for base_2024, add a delta (2025 vs 2024) line on a secondary Y axis, and render a comparative table under the chart. Also include the binary change to data/raw/Retos/Plan de retos.xlsx. Function signatures and return tuples were updated accordingly to propagate the new areas_df.
</commit_message>
<xml_diff>
--- a/data/raw/Retos/Plan de retos.xlsx
+++ b/data/raw/Retos/Plan de retos.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Sistema_Indicadores_Poli/data/raw/Retos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{D4183C01-A731-46D5-A9D4-97CA5D131F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50D4CDDD-03B5-4D19-ADDE-9C48A22123F2}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="8_{D4183C01-A731-46D5-A9D4-97CA5D131F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7C74DB9-D053-415A-99FF-EABDFCDD68C1}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{557E1470-D854-4955-8C66-3C30D44953A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{557E1470-D854-4955-8C66-3C30D44953A5}"/>
   </bookViews>
   <sheets>
     <sheet name="Linea" sheetId="1" r:id="rId1"/>
     <sheet name="Objetivo" sheetId="2" r:id="rId2"/>
     <sheet name="Planes" sheetId="3" r:id="rId3"/>
+    <sheet name="Areas" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="25">
   <si>
     <t>Línea Estratégica</t>
   </si>
@@ -110,6 +111,9 @@
   </si>
   <si>
     <t>N°</t>
+  </si>
+  <si>
+    <t>Desglose</t>
   </si>
 </sst>
 </file>
@@ -343,6 +347,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="13" formatCode="0%"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -594,6 +599,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="13" formatCode="0%"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -773,6 +779,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0D56B507-94F7-45AC-A862-EDB1AC90037F}" name="Tabla3" displayName="Tabla3" ref="A1:E25" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16" totalsRowBorderDxfId="15">
   <autoFilter ref="A1:E25" xr:uid="{0D56B507-94F7-45AC-A862-EDB1AC90037F}"/>
@@ -782,7 +792,7 @@
     <tableColumn id="3" xr3:uid="{D949FAD6-480B-4FDA-9AE8-31D46A8ED7B5}" name="Meta" dataDxfId="12"/>
     <tableColumn id="4" xr3:uid="{7663C50E-80CF-4F20-9587-4EAA4F1B329E}" name="Ejecución" dataDxfId="11" dataCellStyle="Porcentaje"/>
     <tableColumn id="5" xr3:uid="{FA88A2D1-6122-4340-9A57-12F7D7AD2114}" name="Cumplimiento" dataDxfId="10" dataCellStyle="Porcentaje">
-      <calculatedColumnFormula>D2/C2</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(D2/C2&gt;1,1,D2/C2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -790,8 +800,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06F90347-0855-4383-9569-33279D7F9297}" name="Tabla2" displayName="Tabla2" ref="A1:F34" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
-  <autoFilter ref="A1:F34" xr:uid="{06F90347-0855-4383-9569-33279D7F9297}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{06F90347-0855-4383-9569-33279D7F9297}" name="Tabla2" displayName="Tabla2" ref="A1:F45" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+  <autoFilter ref="A1:F45" xr:uid="{06F90347-0855-4383-9569-33279D7F9297}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{22977429-7756-49B9-8F1C-59D1D94ADD97}" name="Línea Estratégica" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{C0147790-F88D-4586-A14D-912D57FA7C78}" name="Objetivo" dataDxfId="4"/>
@@ -799,7 +809,7 @@
     <tableColumn id="4" xr3:uid="{6EC61543-8E4A-4D24-A5D7-28C80DC56C56}" name="Meta" dataDxfId="2"/>
     <tableColumn id="5" xr3:uid="{D180F852-CE12-4DC1-8BBC-10FFE646B4E1}" name="Ejecución" dataDxfId="1"/>
     <tableColumn id="6" xr3:uid="{E7063ED5-D130-42FD-A7A0-2D1D9802D166}" name="Cumplimiento" dataDxfId="0" dataCellStyle="Porcentaje">
-      <calculatedColumnFormula>E2/D2</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(E2/D2&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -807,11 +817,22 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BD1E2EEB-A153-4351-825D-DD31E3D95F4E}" name="Tabla1" displayName="Tabla1" ref="A1:B5" totalsRowShown="0">
-  <autoFilter ref="A1:B5" xr:uid="{BD1E2EEB-A153-4351-825D-DD31E3D95F4E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BD1E2EEB-A153-4351-825D-DD31E3D95F4E}" name="Tabla1" displayName="Tabla1" ref="A1:C25" totalsRowShown="0">
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{FAF0C870-F1EF-4DAF-A0CA-013947A2527F}" name="Año"/>
+    <tableColumn id="3" xr3:uid="{F4222E18-D2D2-4FB1-90CC-28583FE1F728}" name="Desglose"/>
+    <tableColumn id="2" xr3:uid="{F8D852DD-2136-45BD-93C2-DE2432F9011B}" name="N°"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{36859B46-A924-485F-BA67-2AB7CF75A0BD}" name="Tabla4" displayName="Tabla4" ref="A1:B6" totalsRowShown="0">
+  <autoFilter ref="A1:B6" xr:uid="{36859B46-A924-485F-BA67-2AB7CF75A0BD}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{FAF0C870-F1EF-4DAF-A0CA-013947A2527F}" name="Año"/>
-    <tableColumn id="2" xr3:uid="{F8D852DD-2136-45BD-93C2-DE2432F9011B}" name="N°"/>
+    <tableColumn id="1" xr3:uid="{97246F26-F740-47DC-A136-932AD3FF683D}" name="Año"/>
+    <tableColumn id="2" xr3:uid="{D14DD27A-5F2E-4A19-BD94-2116649FC976}" name="N°"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1173,7 +1194,7 @@
         <v>0.99876373626373605</v>
       </c>
       <c r="E2" s="9">
-        <f>D2/C2</f>
+        <f t="shared" ref="E2:E25" si="0">IF(D2/C2&gt;1,1,D2/C2)</f>
         <v>0.99876373626373605</v>
       </c>
       <c r="F2" s="1"/>
@@ -1193,7 +1214,7 @@
         <v>0.99164021164021199</v>
       </c>
       <c r="E3" s="9">
-        <f t="shared" ref="E3:E7" si="0">D3/C3</f>
+        <f t="shared" si="0"/>
         <v>0.99164021164021199</v>
       </c>
       <c r="F3" s="1"/>
@@ -1293,7 +1314,7 @@
         <v>0.98771471471471495</v>
       </c>
       <c r="E8" s="9">
-        <f>D8/C8</f>
+        <f t="shared" si="0"/>
         <v>0.98771471471471495</v>
       </c>
     </row>
@@ -1311,7 +1332,7 @@
         <v>0.96605329457364397</v>
       </c>
       <c r="E9" s="9">
-        <f t="shared" ref="E9:E13" si="1">D9/C9</f>
+        <f t="shared" si="0"/>
         <v>0.96605329457364397</v>
       </c>
     </row>
@@ -1329,7 +1350,7 @@
         <v>0.985607344632768</v>
       </c>
       <c r="E10" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.985607344632768</v>
       </c>
     </row>
@@ -1347,7 +1368,7 @@
         <v>0.97506976744186002</v>
       </c>
       <c r="E11" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.97506976744186002</v>
       </c>
     </row>
@@ -1365,7 +1386,7 @@
         <v>0.98925490196078403</v>
       </c>
       <c r="E12" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.98925490196078403</v>
       </c>
     </row>
@@ -1383,7 +1404,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
@@ -1401,7 +1422,7 @@
         <v>0.97313400900900904</v>
       </c>
       <c r="E14" s="9">
-        <f>D14/C14</f>
+        <f t="shared" si="0"/>
         <v>0.97313400900900904</v>
       </c>
     </row>
@@ -1419,7 +1440,7 @@
         <v>0.98857142857142899</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" ref="E15:E19" si="2">D15/C15</f>
+        <f t="shared" si="0"/>
         <v>0.98857142857142899</v>
       </c>
     </row>
@@ -1437,7 +1458,7 @@
         <v>0.95625170068027199</v>
       </c>
       <c r="E16" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0.95625170068027199</v>
       </c>
     </row>
@@ -1455,7 +1476,7 @@
         <v>0.98229126984127002</v>
       </c>
       <c r="E17" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0.98229126984127002</v>
       </c>
     </row>
@@ -1473,7 +1494,7 @@
         <v>0.96579037800687295</v>
       </c>
       <c r="E18" s="9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0.96579037800687295</v>
       </c>
     </row>
@@ -1490,8 +1511,8 @@
       <c r="D19" s="22">
         <v>0.97948275862069001</v>
       </c>
-      <c r="E19" s="18">
-        <f t="shared" si="2"/>
+      <c r="E19" s="9">
+        <f t="shared" si="0"/>
         <v>0.97948275862069001</v>
       </c>
     </row>
@@ -1509,8 +1530,8 @@
         <v>0.32</v>
       </c>
       <c r="E20" s="9">
-        <f>D20/C20</f>
-        <v>1.1428571428571428</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -1527,8 +1548,8 @@
         <v>0.33</v>
       </c>
       <c r="E21" s="9">
-        <f t="shared" ref="E21:E25" si="3">D21/C21</f>
-        <v>1.03125</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1545,7 +1566,7 @@
         <v>0.28920000000000001</v>
       </c>
       <c r="E22" s="9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>0.95131578947368423</v>
       </c>
     </row>
@@ -1556,11 +1577,15 @@
       <c r="B23" s="2">
         <v>2026</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="9" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+      <c r="C23" s="4">
+        <v>0.31</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0.33</v>
+      </c>
+      <c r="E23" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -1570,11 +1595,15 @@
       <c r="B24" s="2">
         <v>2026</v>
       </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="9" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+      <c r="C24" s="4">
+        <v>0.32</v>
+      </c>
+      <c r="D24" s="6">
+        <v>0.33</v>
+      </c>
+      <c r="E24" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1584,11 +1613,15 @@
       <c r="B25" s="2">
         <v>2026</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="18" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+      <c r="C25" s="16">
+        <v>0.31125000000000003</v>
+      </c>
+      <c r="D25" s="22">
+        <v>0.2472</v>
+      </c>
+      <c r="E25" s="9">
+        <f t="shared" si="0"/>
+        <v>0.79421686746987941</v>
       </c>
     </row>
   </sheetData>
@@ -1601,7 +1634,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9707B1A2-0D04-49F9-B895-08B6833A3BE4}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46.88671875" customWidth="1"/>
@@ -1649,7 +1682,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="9">
-        <f>E2/D2</f>
+        <f>IF(E2/D2&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1670,7 +1703,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="9">
-        <f t="shared" ref="F3:F34" si="0">E3/D3</f>
+        <f>IF(E3/D3&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1691,7 +1724,7 @@
         <v>0.96</v>
       </c>
       <c r="F4" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E4/D4&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.96</v>
       </c>
     </row>
@@ -1712,7 +1745,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E5/D5&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1733,7 +1766,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E6/D6&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1754,7 +1787,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E7/D7&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1775,7 +1808,7 @@
         <v>0.98</v>
       </c>
       <c r="F8" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E8/D8&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.98</v>
       </c>
     </row>
@@ -1796,7 +1829,7 @@
         <v>0.99</v>
       </c>
       <c r="F9" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E9/D9&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.99</v>
       </c>
     </row>
@@ -1817,7 +1850,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E10/D10&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1838,7 +1871,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E11/D11&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1859,7 +1892,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E12/D12&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1880,7 +1913,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E13/D13&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -1901,7 +1934,7 @@
         <v>0.97</v>
       </c>
       <c r="F14" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E14/D14&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.97</v>
       </c>
     </row>
@@ -1922,7 +1955,7 @@
         <v>0.93</v>
       </c>
       <c r="F15" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E15/D15&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.93</v>
       </c>
     </row>
@@ -1943,7 +1976,7 @@
         <v>0.98</v>
       </c>
       <c r="F16" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E16/D16&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.98</v>
       </c>
     </row>
@@ -1964,7 +1997,7 @@
         <v>0.98</v>
       </c>
       <c r="F17" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E17/D17&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.98</v>
       </c>
     </row>
@@ -1985,7 +2018,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E18/D18&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -2006,7 +2039,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E19/D19&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -2027,7 +2060,7 @@
         <v>0.99</v>
       </c>
       <c r="F20" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E20/D20&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.99</v>
       </c>
     </row>
@@ -2048,7 +2081,7 @@
         <v>0.99</v>
       </c>
       <c r="F21" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E21/D21&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.99</v>
       </c>
     </row>
@@ -2069,7 +2102,7 @@
         <v>0.98</v>
       </c>
       <c r="F22" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E22/D22&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.98</v>
       </c>
     </row>
@@ -2090,7 +2123,7 @@
         <v>0.99</v>
       </c>
       <c r="F23" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E23/D23&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.99</v>
       </c>
     </row>
@@ -2111,7 +2144,7 @@
         <v>0.96</v>
       </c>
       <c r="F24" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E24/D24&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.96</v>
       </c>
     </row>
@@ -2132,7 +2165,7 @@
         <v>0.98</v>
       </c>
       <c r="F25" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E25/D25&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.98</v>
       </c>
     </row>
@@ -2153,7 +2186,7 @@
         <v>1</v>
       </c>
       <c r="F26" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E26/D26&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>1</v>
       </c>
     </row>
@@ -2174,7 +2207,7 @@
         <v>0.98</v>
       </c>
       <c r="F27" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E27/D27&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.98</v>
       </c>
     </row>
@@ -2195,7 +2228,7 @@
         <v>0.98</v>
       </c>
       <c r="F28" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E28/D28&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.98</v>
       </c>
     </row>
@@ -2216,7 +2249,7 @@
         <v>0.99</v>
       </c>
       <c r="F29" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E29/D29&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.99</v>
       </c>
     </row>
@@ -2237,7 +2270,7 @@
         <v>0.97</v>
       </c>
       <c r="F30" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E30/D30&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.97</v>
       </c>
     </row>
@@ -2258,7 +2291,7 @@
         <v>0.97</v>
       </c>
       <c r="F31" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E31/D31&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.97</v>
       </c>
     </row>
@@ -2279,7 +2312,7 @@
         <v>0.94</v>
       </c>
       <c r="F32" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E32/D32&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.94</v>
       </c>
     </row>
@@ -2300,7 +2333,7 @@
         <v>0.97</v>
       </c>
       <c r="F33" s="9">
-        <f t="shared" si="0"/>
+        <f>IF(E33/D33&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.97</v>
       </c>
     </row>
@@ -2321,8 +2354,239 @@
         <v>0.93</v>
       </c>
       <c r="F34" s="18">
-        <f t="shared" si="0"/>
+        <f>IF(E34/D34&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
         <v>0.93</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D35" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="E35" s="5">
+        <v>0.33</v>
+      </c>
+      <c r="F35" s="9">
+        <f>IF(E35/D35&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D36" s="4">
+        <v>0.3</v>
+      </c>
+      <c r="E36" s="5">
+        <v>0.312</v>
+      </c>
+      <c r="F36" s="9">
+        <f>IF(E36/D36&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D37" s="4">
+        <v>0.29599999999999999</v>
+      </c>
+      <c r="E37" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="F37" s="9">
+        <f>IF(E37/D37&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D38" s="4">
+        <v>0.33</v>
+      </c>
+      <c r="E38" s="5">
+        <v>0.35</v>
+      </c>
+      <c r="F38" s="9">
+        <f>IF(E38/D38&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D39" s="4">
+        <v>0.31</v>
+      </c>
+      <c r="E39" s="5">
+        <v>0.33</v>
+      </c>
+      <c r="F39" s="9">
+        <f>IF(E39/D39&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D40" s="4">
+        <v>0.252</v>
+      </c>
+      <c r="E40" s="5">
+        <v>0.25</v>
+      </c>
+      <c r="F40" s="9">
+        <f>IF(E40/D40&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>0.99206349206349209</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D41" s="4">
+        <v>0.315</v>
+      </c>
+      <c r="E41" s="5">
+        <v>0.25</v>
+      </c>
+      <c r="F41" s="9">
+        <f>IF(E41/D41&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>0.79365079365079361</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D42" s="4">
+        <v>0.32</v>
+      </c>
+      <c r="E42" s="5">
+        <v>0.33</v>
+      </c>
+      <c r="F42" s="9">
+        <f>IF(E42/D42&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C43" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D43" s="4">
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="E43" s="5">
+        <v>0.216</v>
+      </c>
+      <c r="F43" s="9">
+        <f>IF(E43/D43&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>0.82442748091603046</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D44" s="4">
+        <v>0.35</v>
+      </c>
+      <c r="E44" s="5">
+        <v>0.38</v>
+      </c>
+      <c r="F44" s="9">
+        <f>IF(E44/D44&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C45" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D45" s="16">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="E45" s="17">
+        <v>0.218</v>
+      </c>
+      <c r="F45" s="18">
+        <f>IF(E45/D45&gt;1,1,Tabla2[[#This Row],[Ejecución]]/Tabla2[[#This Row],[Meta]])</f>
+        <v>0.77857142857142847</v>
       </c>
     </row>
   </sheetData>
@@ -2335,8 +2599,297 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{450245B9-0154-498C-A9D0-E79BCBDD5F55}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2023</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2023</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2023</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2023</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2023</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2024</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2024</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>2024</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>2024</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>2024</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>2024</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2025</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2025</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2025</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2025</v>
+      </c>
+      <c r="B17" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2025</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2025</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2026</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>2026</v>
+      </c>
+      <c r="B21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2026</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2026</v>
+      </c>
+      <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2026</v>
+      </c>
+      <c r="B24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2026</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFEF2421-346E-4A38-9990-7BD73E815025}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -2376,6 +2929,14 @@
       </c>
       <c r="B5">
         <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2026</v>
+      </c>
+      <c r="B6">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>